<commit_message>
feat(F-NAR-016): TREE-DIF-055 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-055.xlsx
+++ b/stories/arbres/TREE-DIF-055.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La casserole a laissé un nuage sur la vitre. Les carreaux sont encore un peu froids. Ça sent le toast d'avant, tout tiède. Une goutte glisse, lente, sur le carreau. Le citron est là, Sarah, tu le vois ? Il est tout jaune, papa. Maman pose le pichet bleu près de l'eau. On fait une citronnade, tu veux ? Oui, tout un pichet ! En ce moment, Sarah touche le citron. Je le roule, il est froid. Merci, tu le tiens tout droit. Le sucrier aussi, tout près. On prépare, alors ?</t>
+          <t>La casserole a laissé un nuage sur la vitre. Les carreaux sont encore un peu froids. Tu as froid aux pieds, Sarah ? Un peu, papa. Ça sent le toast d'avant, tout tiède. Une goutte glisse, lente, sur le carreau. Le citron est là, tu le vois ? Il est tout jaune, papa. Maman pose le pichet bleu près de l'eau. On fait une citronnade, tu veux ? Oui, tout un pichet ! En ce moment, Sarah touche le citron. Je le roule, il est froid. Merci, tu le tiens tout droit. Le sucrier aussi, tout près. On prépare, alors ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La casserole a laissé un nuage sur la vitre. Les carreaux sont encore un peu froids. Ça sent le toast d'avant, tout tiède. Une goutte glisse, lente, sur le carreau. Le citron est là, Sarah, tu le vois ? Il est tout jaune, papa. Maman pose le pichet bleu près de l'eau. On fait une citronnade, tu veux ? Oui, tout un pichet ! En ce moment, Sarah touche le citron. Je le roule, il est froid. Merci, tu le tiens tout droit. Le sucrier aussi, tout près. On prépare, alors ?</t>
+          <t>La casserole a laissé un nuage sur la vitre. Les carreaux sont encore un peu froids. Tu as froid aux pieds, Sarah ? Un peu, papa. Ça sent le toast d'avant, tout tiède. Une goutte glisse, lente, sur le carreau. Le citron est là, tu le vois ? Il est tout jaune, papa. Maman pose le pichet bleu près de l'eau. On fait une citronnade, tu veux ? Oui, tout un pichet ! En ce moment, Sarah touche le citron. Je le roule, il est froid. Merci, tu le tiens tout droit. Le sucrier aussi, tout près. On prépare, alors ?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1339,9 +1339,11 @@
         <is>
           <t>narrateur|La casserole a laissé un nuage sur la vitre.
 narrateur|Les carreaux sont encore un peu froids.
+papa|Tu as froid aux pieds, Sarah ?
+enfant-f|Un peu, papa.
 narrateur|Ça sent le toast d'avant, tout tiède.
 narrateur|Une goutte glisse, lente, sur le carreau.
-papa|Le citron est là, Sarah, tu le vois ?
+papa|Le citron est là, tu le vois ?
 enfant-f|Il est tout jaune, papa.
 narrateur|Maman pose le pichet bleu près de l'eau.
 maman|On fait une citronnade, tu veux ?
@@ -1570,12 +1572,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord le citron jaune. Il est froid, tout rond. Garde-le dans les mains, tout droit. La peau sent déjà le soleil. Le sucrier aussi, près de toi. Maman glisse le pichet, tout près. Les trois affaires avancent avec elle. La citronnade va venir. Ses pieds tapent déjà le carreau, trop vite. Le citron d'abord, vous l'avez.</t>
+          <t>Sarah prend d'abord le citron jaune. Il est froid, tout rond. Garde-le dans les mains, tout droit. La peau sent déjà le soleil. Le sucrier aussi, près de toi. Maman glisse le pichet, tout près. Citron, sucrier, pichet, tout contre elle. La citronnade va venir. Ses pieds tapent déjà le carreau, trop vite. Le citron d'abord, vous l'avez.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord le citron jaune. Il est froid, tout rond. Garde-le dans les mains, tout droit. La peau sent déjà le soleil. Le sucrier aussi, près de toi. Maman glisse le pichet, tout près. Les trois affaires avancent avec elle. La citronnade va venir. Ses pieds tapent déjà le carreau, trop vite. Le citron d'abord, vous l'avez.</t>
+          <t>Sarah prend d'abord le citron jaune. Il est froid, tout rond. Garde-le dans les mains, tout droit. La peau sent déjà le soleil. Le sucrier aussi, près de toi. Maman glisse le pichet, tout près. Citron, sucrier, pichet, tout contre elle. La citronnade va venir. Ses pieds tapent déjà le carreau, trop vite. Le citron d'abord, vous l'avez.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1716,7 +1718,7 @@
 narrateur|La peau sent déjà le soleil.
 papa|Le sucrier aussi, près de toi.
 narrateur|Maman glisse le pichet, tout près.
-narrateur|Les trois affaires avancent avec elle.
+narrateur|Citron, sucrier, pichet, tout contre elle.
 enfant-f|La citronnade va venir.
 narrateur|Ses pieds tapent déjà le carreau, trop vite.
 papa|Le citron d'abord, vous l'avez.</t>
@@ -2304,12 +2306,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le citron sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le citron part, comme une petite balle. Le citron jaune part trop vite. Tes pieds dansent, déjà. La table n'a pas encore de jus. On presse comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Sarah pose le citron sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le citron part, comme une petite balle. Le citron jaune part trop vite. Tes pieds dansent, déjà. Le jus n'est pas encore là. On presse comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le citron sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le citron part, comme une petite balle. Le citron jaune part trop vite. Tes pieds dansent, déjà. La table n'a pas encore de jus. On presse comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Sarah pose le citron sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le citron part, comme une petite balle. Le citron jaune part trop vite. Tes pieds dansent, déjà. Le jus n'est pas encore là. On presse comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2450,7 +2452,7 @@
 narrateur|Le citron part, comme une petite balle.
 enfant-f|Le citron jaune part trop vite.
 maman|Tes pieds dansent, déjà.
-papa|La table n'a pas encore de jus.
+papa|Le jus n'est pas encore là.
 enfant-f|On presse comment, alors ?
 papa|Tu fais comment, avec nous ?</t>
         </is>
@@ -2671,12 +2673,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule le citron, un, deux, trois. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Vous avez joué, puis posé. La toile redevient une table, tout douce.</t>
+          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule le citron, un, deux, trois. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Le jus tombe dans le pichet, tout jaune. Tu as roulé, moi j'ai rattrapé. La toile redevient une table, tout douce.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule le citron, un, deux, trois. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Vous avez joué, puis posé. La toile redevient une table, tout douce.</t>
+          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule le citron, un, deux, trois. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Le jus tombe dans le pichet, tout jaune. Tu as roulé, moi j'ai rattrapé. La toile redevient une table, tout douce.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2818,7 +2820,8 @@
 narrateur|Sarah roule encore, puis s'arrête.
 enfant-f|La balle est fatiguée.
 maman|On peut presser, maintenant.
-papa|Vous avez joué, puis posé.
+narrateur|Le jus tombe dans le pichet, tout jaune.
+papa|Tu as roulé, moi j'ai rattrapé.
 narrateur|La toile redevient une table, tout douce.</t>
         </is>
       </c>
@@ -2846,12 +2849,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le citron jaune garde une peau froide, tout près. Un grain sucré dort sur la toile. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
+          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le citron jaune garde une peau froide, tout près. Sarah lèche une goutte sur le bord. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le citron jaune garde une peau froide, tout près. Un grain sucré dort sur la toile. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
+          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le citron jaune garde une peau froide, tout près. Sarah lèche une goutte sur le bord. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2992,7 +2995,7 @@
 maman|Le pichet a son jaune, maintenant.
 narrateur|La toile cirée garde un grain sucré.
 narrateur|Le citron jaune garde une peau froide, tout près.
-narrateur|Un grain sucré dort sur la toile.
+narrateur|Sarah lèche une goutte sur le bord.
 enfant-f|Encore une gorgée, papa.
 narrateur|La vitre tient encore le soleil.</t>
         </is>
@@ -3021,12 +3024,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>On attend le grain. Sarah pose les genoux au carreau. Le citron repose, enfin sage. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. La citronnade peut venir.</t>
+          <t>On attend le grain. Sarah pose les genoux au carreau. Le citron repose, enfin sage. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. Le jus tombe, une goutte, puis deux. La citronnade peut venir.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>On attend le grain. Sarah pose les genoux au carreau. Le citron repose, enfin sage. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. La citronnade peut venir.</t>
+          <t>On attend le grain. Sarah pose les genoux au carreau. Le citron repose, enfin sage. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. Le jus tombe, une goutte, puis deux. La citronnade peut venir.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3169,6 +3172,7 @@
 maman|La toile est calme, oui.
 papa|Tes pieds se sont assis, eux aussi.
 narrateur|Sarah presse, tout droit, tout petit.
+narrateur|Le jus tombe, une goutte, puis deux.
 enfant-f|La citronnade peut venir.</t>
         </is>
       </c>
@@ -3371,12 +3375,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le citron, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Vous avez demandé, et ça tient. Ma main fait le bol, ici. La table garde un grain, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le citron, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Le jus rejoint le sucre, tout jaune. Ma main tient, la tienne verse. La table garde un grain, tout mince.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le citron, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Vous avez demandé, et ça tient. Ma main fait le bol, ici. La table garde un grain, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le citron, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Le jus rejoint le sucre, tout jaune. Ma main tient, la tienne verse. La table garde un grain, tout mince.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3517,8 +3521,8 @@
 narrateur|Sarah verse un grain, puis un autre.
 narrateur|Le jaune reste sage, dans sa main.
 enfant-f|Toi tu tiens, moi je verse.
-papa|Vous avez demandé, et ça tient.
-maman|Ma main fait le bol, ici.
+narrateur|Le jus rejoint le sucre, tout jaune.
+maman|Ma main tient, la tienne verse.
 narrateur|La table garde un grain, tout mince.</t>
         </is>
       </c>
@@ -3546,12 +3550,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Vous avez demandé, et ça tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le citron jaune pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
+          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Tu demandais, maman tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le citron jaune pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Vous avez demandé, et ça tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le citron jaune pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
+          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Tu demandais, maman tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le citron jaune pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3688,7 +3692,7 @@
         <is>
           <t>narrateur|Sarah boit, la main de maman tout près.
 enfant-f|Tu tenais le fruit.
-papa|Vous avez demandé, et ça tenait.
+papa|Tu demandais, maman tenait.
 maman|Ma main a fait le bol.
 narrateur|La cuisine rend le silence, tout doux.
 narrateur|Le citron jaune pose un grain de lumière.
@@ -3721,12 +3725,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le citron vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le citron glisse, trop mouillé, trop vite. Une goutte rebondit, puis s'en va. Ton corps veut encore courir. L'évier n'a pas encore de pichet. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah porte le citron vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le citron glisse, trop mouillé, trop vite. Une goutte rebondit, puis s'en va. Tes genoux rebondissent encore. Le pichet n'a pas encore de jus. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le citron vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le citron glisse, trop mouillé, trop vite. Une goutte rebondit, puis s'en va. Ton corps veut encore courir. L'évier n'a pas encore de pichet. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah porte le citron vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le citron glisse, trop mouillé, trop vite. Une goutte rebondit, puis s'en va. Tes genoux rebondissent encore. Le pichet n'a pas encore de jus. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3866,8 +3870,8 @@
 narrateur|Ses genoux font un petit trampoline.
 narrateur|Le citron glisse, trop mouillé, trop vite.
 narrateur|Une goutte rebondit, puis s'en va.
-maman|Ton corps veut encore courir.
-papa|L'évier n'a pas encore de pichet.
+maman|Tes genoux rebondissent encore.
+papa|Le pichet n'a pas encore de jus.
 enfant-f|On peut jouer avec, quand même ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -4088,12 +4092,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah presse, papa compte les gouttes. Des perles tombent, une après l'autre. La dernière est au bout. Vous avez joué, puis posé le fruit. L'évier est devenu un ruisseau. Le citron jaune a trouvé son coin. Le jus est là, tout bas.</t>
+          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah presse, papa compte les gouttes. Des perles tombent, une après l'autre. La dernière est au bout. Le pichet se teinte, tout doucement. L'évier est devenu un ruisseau. Le citron jaune reste près de l'eau. Le jus est là, tout bas.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah presse, papa compte les gouttes. Des perles tombent, une après l'autre. La dernière est au bout. Vous avez joué, puis posé le fruit. L'évier est devenu un ruisseau. Le citron jaune a trouvé son coin. Le jus est là, tout bas.</t>
+          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah presse, papa compte les gouttes. Des perles tombent, une après l'autre. La dernière est au bout. Le pichet se teinte, tout doucement. L'évier est devenu un ruisseau. Le citron jaune reste près de l'eau. Le jus est là, tout bas.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4233,9 +4237,9 @@
 narrateur|Sarah presse, papa compte les gouttes.
 narrateur|Des perles tombent, une après l'autre.
 enfant-f|La dernière est au bout.
-maman|Vous avez joué, puis posé le fruit.
+narrateur|Le pichet se teinte, tout doucement.
 papa|L'évier est devenu un ruisseau.
-narrateur|Le citron jaune a trouvé son coin.
+narrateur|Le citron jaune reste près de l'eau.
 enfant-f|Le jus est là, tout bas.</t>
         </is>
       </c>
@@ -4438,12 +4442,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>J'attends le filet. Moi je l'ouvre, puis c'est toi. Sarah tient le citron, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y glisse le citron. Chacun son tour, sur l'évier. Le filet se tait, enfin.</t>
+          <t>J'attends le filet. Moi j'ouvre un peu, puis c'est toi. Sarah tient le citron, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y verse le jaune. D'abord l'eau, ensuite le citron. Le filet se tait, enfin.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>J'attends le filet. Moi je l'ouvre, puis c'est toi. Sarah tient le citron, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y glisse le citron. Chacun son tour, sur l'évier. Le filet se tait, enfin.</t>
+          <t>J'attends le filet. Moi j'ouvre un peu, puis c'est toi. Sarah tient le citron, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y verse le jaune. D'abord l'eau, ensuite le citron. Le filet se tait, enfin.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4579,13 +4583,13 @@
       <c r="AW20" t="inlineStr">
         <is>
           <t>enfant-f|J'attends le filet.
-papa|Moi je l'ouvre, puis c'est toi.
+papa|Moi j'ouvre un peu, puis c'est toi.
 narrateur|Sarah tient le citron, le filet attend.
 narrateur|L'eau avance, goutte après goutte.
 narrateur|Sarah souffle, les épaules baissent.
 papa|C'est à toi, Sarah.
-enfant-f|J'y glisse le citron.
-maman|Chacun son tour, sur l'évier.
+enfant-f|J'y verse le jaune.
+maman|D'abord l'eau, ensuite le citron.
 narrateur|Le filet se tait, enfin.</t>
         </is>
       </c>
@@ -4613,12 +4617,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. Chacun son tour, sur l'évier. Le pichet bleu tient, enfin. Le citron jaune garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
+          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. D'abord l'eau, ensuite le jaune. Le pichet bleu tient, enfin. Le citron jaune garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. Chacun son tour, sur l'évier. Le pichet bleu tient, enfin. Le citron jaune garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
+          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. D'abord l'eau, ensuite le jaune. Le pichet bleu tient, enfin. Le citron jaune garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4756,7 +4760,7 @@
           <t>narrateur|Sarah boit, le filet tout calme.
 papa|J'ai ouvert, puis c'était toi.
 enfant-f|J'ai attendu l'eau.
-maman|Chacun son tour, sur l'évier.
+maman|D'abord l'eau, ensuite le jaune.
 narrateur|Le pichet bleu tient, enfin.
 narrateur|Le citron jaune garde un grain de lumière.
 narrateur|Sarah souffle dessus, tout doux.
@@ -4788,12 +4792,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse le citron, tout doux. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Vous avez demandé, et ça marche. Le jus tient tout seul, maintenant. Un carré de carreau reste tiède, autour.</t>
+          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse le citron, tout doux. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Le jaune tombe, le pichet se remplit. Le jus tient tout seul, maintenant. Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse le citron, tout doux. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Vous avez demandé, et ça marche. Le jus tient tout seul, maintenant. Un carré de carreau reste tiède, autour.</t>
+          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse le citron, tout doux. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Le jaune tombe, le pichet se remplit. Le jus tient tout seul, maintenant. Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4934,9 +4938,9 @@
 narrateur|Sarah glisse un grain, les mains calmes.
 narrateur|L'autre main suit, le pichet au calme.
 enfant-f|Toi tu presses, moi je verse.
-maman|Vous avez demandé, et ça marche.
+narrateur|Le jaune tombe, le pichet se remplit.
 papa|Le jus tient tout seul, maintenant.
-narrateur|Un carré de carreau reste tiède, autour.</t>
+narrateur|Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
     </row>
@@ -4963,12 +4967,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. L'entrée du pichet est à vous. L'évier a rendu le calme. Le citron jaune garde une peau froide, tout près. Un rond de chaleur reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
+          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. Le pichet a son jaune, à vous. L'évier a rendu le calme. Le citron jaune garde une peau froide, tout près. Un rond d'eau reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. L'entrée du pichet est à vous. L'évier a rendu le calme. Le citron jaune garde une peau froide, tout près. Un rond de chaleur reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
+          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. Le pichet a son jaune, à vous. L'évier a rendu le calme. Le citron jaune garde une peau froide, tout près. Un rond d'eau reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5106,10 +5110,10 @@
           <t>narrateur|Sarah boit, le citron pressé par papa.
 enfant-f|Tu pressais, tout doux.
 papa|Le jus est tombé, juste assez.
-maman|L'entrée du pichet est à vous.
+maman|Le pichet a son jaune, à vous.
 narrateur|L'évier a rendu le calme.
 narrateur|Le citron jaune garde une peau froide, tout près.
-narrateur|Un rond de chaleur reste sur le carreau.
+narrateur|Un rond d'eau reste sur le carreau.
 enfant-f|Regarde, papa, il brille.
 narrateur|Une odeur de citron reste, au frais.</t>
         </is>
@@ -5138,12 +5142,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Sarah grimpe, le citron contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le citron saute d'un genou, trop haut. Le citron jaune n'est plus à sa place. Tes genoux font trop de vagues. Le tabouret n'a pas encore de table. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah grimpe, le citron contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le citron saute d'un genou, trop haut. Le citron jaune n'est plus à sa place. Tes genoux font trop de vagues. Le jus n'est pas encore versé. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sarah grimpe, le citron contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le citron saute d'un genou, trop haut. Le citron jaune n'est plus à sa place. Tes genoux font trop de vagues. Le tabouret n'a pas encore de table. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah grimpe, le citron contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le citron saute d'un genou, trop haut. Le citron jaune n'est plus à sa place. Tes genoux font trop de vagues. Le jus n'est pas encore versé. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5284,7 +5288,7 @@
 narrateur|Le citron saute d'un genou, trop haut.
 narrateur|Le citron jaune n'est plus à sa place.
 maman|Tes genoux font trop de vagues.
-papa|Le tabouret n'a pas encore de table.
+papa|Le jus n'est pas encore versé.
 enfant-f|On verse comment, alors ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -5505,12 +5509,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>On fait des sauts. Tu rebondis, puis tu verses. Le citron voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Vous avez joué, puis versé. Le tabouret est une table, maintenant. Le citron jaune a trouvé son coin. La citronnade est là, tout haut.</t>
+          <t>On fait des sauts. Tu rebondis, puis tu verses. Le citron voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Sarah verse, le pichet se teinte. Le tabouret est une table, maintenant. Le citron jaune reste tout près, en haut. La citronnade est là, tout haut.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>On fait des sauts. Tu rebondis, puis tu verses. Le citron voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Vous avez joué, puis versé. Le tabouret est une table, maintenant. Le citron jaune a trouvé son coin. La citronnade est là, tout haut.</t>
+          <t>On fait des sauts. Tu rebondis, puis tu verses. Le citron voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Sarah verse, le pichet se teinte. Le tabouret est une table, maintenant. Le citron jaune reste tout près, en haut. La citronnade est là, tout haut.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5650,9 +5654,9 @@
 narrateur|Le citron voyage d'un genou à l'autre.
 narrateur|Le bois penche, puis se tient droit.
 enfant-f|Doucement, les sauts tiennent.
-maman|Vous avez joué, puis versé.
+narrateur|Sarah verse, le pichet se teinte.
 papa|Le tabouret est une table, maintenant.
-narrateur|Le citron jaune a trouvé son coin.
+narrateur|Le citron jaune reste tout près, en haut.
 enfant-f|La citronnade est là, tout haut.</t>
         </is>
       </c>
@@ -5855,12 +5859,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le citron reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Le tabouret a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
+          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le citron reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Sarah verse, une goutte, puis l'eau. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le citron reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Le tabouret a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
+          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le citron reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Sarah verse, une goutte, puis l'eau. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -6001,7 +6005,7 @@
 narrateur|Le citron reste sage, au creux des mains.
 narrateur|Le compte se tait, enfin.
 enfant-f|Maintenant !
-maman|Le tabouret a fini ses vagues.
+narrateur|Sarah verse, une goutte, puis l'eau.
 papa|Tes genoux se sont assis, eux aussi.
 narrateur|Un pli du torchon retombe, tout lent.</t>
         </is>
@@ -6205,12 +6209,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu portes le pichet ? Je le porte, tout chaud. Papa porte le pichet, Sarah tient le citron. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le tabouret devient une table, tout haut. Vous avez demandé le bord. Ses mains ont tenu le jaune.</t>
+          <t>Papa, tu portes le pichet ? Je le porte, tout droit. Papa porte le pichet, Sarah tient le citron. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le jaune tombe, vu d'en haut. Tu as demandé, je porte. Tes mains ont tenu le bord.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu portes le pichet ? Je le porte, tout chaud. Papa porte le pichet, Sarah tient le citron. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le tabouret devient une table, tout haut. Vous avez demandé le bord. Ses mains ont tenu le jaune.</t>
+          <t>Papa, tu portes le pichet ? Je le porte, tout droit. Papa porte le pichet, Sarah tient le citron. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le jaune tombe, vu d'en haut. Tu as demandé, je porte. Tes mains ont tenu le bord.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6346,14 +6350,14 @@
       <c r="AW30" t="inlineStr">
         <is>
           <t>enfant-f|Papa, tu portes le pichet ?
-papa|Je le porte, tout chaud.
+papa|Je le porte, tout droit.
 narrateur|Papa porte le pichet, Sarah tient le citron.
 narrateur|Sarah écoute les mains, plus que ses pieds.
 maman|Tu verses, et ça tient.
 enfant-f|Moi aussi, j'écoute.
-narrateur|Le tabouret devient une table, tout haut.
-papa|Vous avez demandé le bord.
-maman|Ses mains ont tenu le jaune.</t>
+narrateur|Le jaune tombe, vu d'en haut.
+papa|Tu as demandé, je porte.
+maman|Tes mains ont tenu le bord.</t>
         </is>
       </c>
     </row>
@@ -6380,12 +6384,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Vous avez demandé le bord. Le tabouret a rendu vos pas. Le citron jaune garde une peau froide, tout près. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
+          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Tu as demandé, il a porté. Le tabouret a rendu vos pas. Le citron jaune garde une peau froide, tout près. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Vous avez demandé le bord. Le tabouret a rendu vos pas. Le citron jaune garde une peau froide, tout près. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
+          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Tu as demandé, il a porté. Le tabouret a rendu vos pas. Le citron jaune garde une peau froide, tout près. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6523,7 +6527,7 @@
           <t>narrateur|Sarah boit, le pichet porté par papa.
 enfant-f|J'écoutais tes mains.
 papa|Moi aussi, je portais avec toi.
-maman|Vous avez demandé le bord.
+maman|Tu as demandé, il a porté.
 narrateur|Le tabouret a rendu vos pas.
 narrateur|Le citron jaune garde une peau froide, tout près.
 narrateur|Sarah touche le verre, du bout des doigts.
@@ -6555,12 +6559,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Sarah serre d'abord le sucrier blanc. Il gratte un peu, contre moi. Tiens-le contre le ventre, tout chaud. Un grain tombe, tout petit. Le citron, ensuite, près de toi. Elle glisse le pichet d'une main. Les trois affaires avancent avec elle. Je veux le jus, tout jaune. Un genou rebondit, puis l'autre. Le sucrier d'abord, il est prêt.</t>
+          <t>Sarah serre d'abord le sucrier blanc. Il gratte un peu, contre moi. Tiens-le contre le ventre, tout chaud. Un grain tombe, tout petit. Le citron, ensuite, près de toi. Elle glisse le pichet d'une main. Le blanc, le jaune, et le bleu. Je veux le jus, tout jaune. Un genou rebondit, puis l'autre. Le sucrier d'abord, il est prêt.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Sarah serre d'abord le sucrier blanc. Il gratte un peu, contre moi. Tiens-le contre le ventre, tout chaud. Un grain tombe, tout petit. Le citron, ensuite, près de toi. Elle glisse le pichet d'une main. Les trois affaires avancent avec elle. Je veux le jus, tout jaune. Un genou rebondit, puis l'autre. Le sucrier d'abord, il est prêt.</t>
+          <t>Sarah serre d'abord le sucrier blanc. Il gratte un peu, contre moi. Tiens-le contre le ventre, tout chaud. Un grain tombe, tout petit. Le citron, ensuite, près de toi. Elle glisse le pichet d'une main. Le blanc, le jaune, et le bleu. Je veux le jus, tout jaune. Un genou rebondit, puis l'autre. Le sucrier d'abord, il est prêt.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -6701,7 +6705,7 @@
 narrateur|Un grain tombe, tout petit.
 maman|Le citron, ensuite, près de toi.
 narrateur|Elle glisse le pichet d'une main.
-narrateur|Les trois affaires avancent avec elle.
+narrateur|Le blanc, le jaune, et le bleu.
 enfant-f|Je veux le jus, tout jaune.
 narrateur|Un genou rebondit, puis l'autre.
 maman|Le sucrier d'abord, il est prêt.</t>
@@ -7289,12 +7293,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le sucrier sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Un grain de sucre saute, trop loin. Le sucrier blanc part trop vite. Tes pieds dansent, déjà. La table n'a pas encore de jus. On presse comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Sarah pose le sucrier sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Un grain de sucre saute, trop loin. Le sucrier blanc part trop vite. Tes pieds dansent, déjà. Le jus n'est pas encore là. On presse comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le sucrier sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Un grain de sucre saute, trop loin. Le sucrier blanc part trop vite. Tes pieds dansent, déjà. La table n'a pas encore de jus. On presse comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Sarah pose le sucrier sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Un grain de sucre saute, trop loin. Le sucrier blanc part trop vite. Tes pieds dansent, déjà. Le jus n'est pas encore là. On presse comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7435,7 +7439,7 @@
 narrateur|Un grain de sucre saute, trop loin.
 enfant-f|Le sucrier blanc part trop vite.
 maman|Tes pieds dansent, déjà.
-papa|La table n'a pas encore de jus.
+papa|Le jus n'est pas encore là.
 enfant-f|On presse comment, alors ?
 papa|Tu fais comment, avec nous ?</t>
         </is>
@@ -7656,12 +7660,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le sucrier devient une colline. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Vous avez joué, puis posé. La toile redevient une table, tout douce.</t>
+          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le sucrier devient une colline. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Le jus tombe dans le pichet, tout jaune. Tu as roulé, moi j'ai rattrapé. La toile redevient une table, tout douce.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le sucrier devient une colline. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Vous avez joué, puis posé. La toile redevient une table, tout douce.</t>
+          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le sucrier devient une colline. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Le jus tombe dans le pichet, tout jaune. Tu as roulé, moi j'ai rattrapé. La toile redevient une table, tout douce.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7803,7 +7807,8 @@
 narrateur|Sarah roule encore, puis s'arrête.
 enfant-f|La balle est fatiguée.
 maman|On peut presser, maintenant.
-papa|Vous avez joué, puis posé.
+narrateur|Le jus tombe dans le pichet, tout jaune.
+papa|Tu as roulé, moi j'ai rattrapé.
 narrateur|La toile redevient une table, tout douce.</t>
         </is>
       </c>
@@ -7831,12 +7836,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le sucrier blanc garde un grain, au fond. Un grain sucré dort sur la toile. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
+          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le sucrier blanc garde un grain, au fond. Sarah lèche une goutte sur le bord. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le sucrier blanc garde un grain, au fond. Un grain sucré dort sur la toile. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
+          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le sucrier blanc garde un grain, au fond. Sarah lèche une goutte sur le bord. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7977,7 +7982,7 @@
 maman|Le pichet a son jaune, maintenant.
 narrateur|La toile cirée garde un grain sucré.
 narrateur|Le sucrier blanc garde un grain, au fond.
-narrateur|Un grain sucré dort sur la toile.
+narrateur|Sarah lèche une goutte sur le bord.
 enfant-f|Encore une gorgée, papa.
 narrateur|La vitre tient encore le soleil.</t>
         </is>
@@ -8006,12 +8011,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>On attend le grain. Sarah pose les genoux au carreau. Le sucrier repose, un grain arrêté. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. La citronnade peut venir.</t>
+          <t>On attend le grain. Sarah pose les genoux au carreau. Le sucrier repose, un grain arrêté. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. Le jus tombe, une goutte, puis deux. La citronnade peut venir.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>On attend le grain. Sarah pose les genoux au carreau. Le sucrier repose, un grain arrêté. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. La citronnade peut venir.</t>
+          <t>On attend le grain. Sarah pose les genoux au carreau. Le sucrier repose, un grain arrêté. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. Le jus tombe, une goutte, puis deux. La citronnade peut venir.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8154,6 +8159,7 @@
 maman|La toile est calme, oui.
 papa|Tes pieds se sont assis, eux aussi.
 narrateur|Sarah presse, tout droit, tout petit.
+narrateur|Le jus tombe, une goutte, puis deux.
 enfant-f|La citronnade peut venir.</t>
         </is>
       </c>
@@ -8356,12 +8362,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le sucrier, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Vous avez demandé, et ça tient. Ma main fait le bol, ici. La table garde un grain, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le sucrier, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Le jus rejoint le sucre, tout jaune. Ma main tient, la tienne verse. La table garde un grain, tout mince.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le sucrier, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Vous avez demandé, et ça tient. Ma main fait le bol, ici. La table garde un grain, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le sucrier, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Le jus rejoint le sucre, tout jaune. Ma main tient, la tienne verse. La table garde un grain, tout mince.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8502,8 +8508,8 @@
 narrateur|Sarah verse un grain, puis un autre.
 narrateur|Le jaune reste sage, dans sa main.
 enfant-f|Toi tu tiens, moi je verse.
-papa|Vous avez demandé, et ça tient.
-maman|Ma main fait le bol, ici.
+narrateur|Le jus rejoint le sucre, tout jaune.
+maman|Ma main tient, la tienne verse.
 narrateur|La table garde un grain, tout mince.</t>
         </is>
       </c>
@@ -8531,12 +8537,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Vous avez demandé, et ça tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le sucrier blanc pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
+          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Tu demandais, maman tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le sucrier blanc pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Vous avez demandé, et ça tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le sucrier blanc pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
+          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Tu demandais, maman tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le sucrier blanc pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8673,7 +8679,7 @@
         <is>
           <t>narrateur|Sarah boit, la main de maman tout près.
 enfant-f|Tu tenais le fruit.
-papa|Vous avez demandé, et ça tenait.
+papa|Tu demandais, maman tenait.
 maman|Ma main a fait le bol.
 narrateur|La cuisine rend le silence, tout doux.
 narrateur|Le sucrier blanc pose un grain de lumière.
@@ -8706,12 +8712,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le sucrier vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le sucrier penche, un grain file. Une goutte rebondit, puis s'en va. Ton corps veut encore courir. L'évier n'a pas encore de pichet. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah porte le sucrier vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le sucrier penche, un grain file. Une goutte rebondit, puis s'en va. Tes genoux rebondissent encore. Le pichet n'a pas encore de jus. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le sucrier vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le sucrier penche, un grain file. Une goutte rebondit, puis s'en va. Ton corps veut encore courir. L'évier n'a pas encore de pichet. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah porte le sucrier vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le sucrier penche, un grain file. Une goutte rebondit, puis s'en va. Tes genoux rebondissent encore. Le pichet n'a pas encore de jus. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8851,8 +8857,8 @@
 narrateur|Ses genoux font un petit trampoline.
 narrateur|Le sucrier penche, un grain file.
 narrateur|Une goutte rebondit, puis s'en va.
-maman|Ton corps veut encore courir.
-papa|L'évier n'a pas encore de pichet.
+maman|Tes genoux rebondissent encore.
+papa|Le pichet n'a pas encore de jus.
 enfant-f|On peut jouer avec, quand même ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -9073,12 +9079,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le sucrier, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Vous avez joué, puis posé le fruit. L'évier est devenu un ruisseau. Le sucrier blanc a trouvé son coin. Le jus est là, tout bas.</t>
+          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le sucrier, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Le pichet se teinte, tout doucement. L'évier est devenu un ruisseau. Le sucrier blanc reste près de l'eau. Le jus est là, tout bas.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le sucrier, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Vous avez joué, puis posé le fruit. L'évier est devenu un ruisseau. Le sucrier blanc a trouvé son coin. Le jus est là, tout bas.</t>
+          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le sucrier, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Le pichet se teinte, tout doucement. L'évier est devenu un ruisseau. Le sucrier blanc reste près de l'eau. Le jus est là, tout bas.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9218,9 +9224,9 @@
 narrateur|Sarah penche le sucrier, papa compte.
 narrateur|Des perles tombent, une après l'autre.
 enfant-f|La dernière est au bout.
-maman|Vous avez joué, puis posé le fruit.
+narrateur|Le pichet se teinte, tout doucement.
 papa|L'évier est devenu un ruisseau.
-narrateur|Le sucrier blanc a trouvé son coin.
+narrateur|Le sucrier blanc reste près de l'eau.
 enfant-f|Le jus est là, tout bas.</t>
         </is>
       </c>
@@ -9423,12 +9429,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>J'attends le filet. Moi je l'ouvre, puis c'est toi. Sarah tient le sucrier, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y glisse le citron. Chacun son tour, sur l'évier. Le filet se tait, enfin.</t>
+          <t>J'attends le filet. Moi j'ouvre un peu, puis c'est toi. Sarah tient le sucrier, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y verse le jaune. D'abord l'eau, ensuite le citron. Le filet se tait, enfin.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J'attends le filet. Moi je l'ouvre, puis c'est toi. Sarah tient le sucrier, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y glisse le citron. Chacun son tour, sur l'évier. Le filet se tait, enfin.</t>
+          <t>J'attends le filet. Moi j'ouvre un peu, puis c'est toi. Sarah tient le sucrier, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y verse le jaune. D'abord l'eau, ensuite le citron. Le filet se tait, enfin.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9564,13 +9570,13 @@
       <c r="AW48" t="inlineStr">
         <is>
           <t>enfant-f|J'attends le filet.
-papa|Moi je l'ouvre, puis c'est toi.
+papa|Moi j'ouvre un peu, puis c'est toi.
 narrateur|Sarah tient le sucrier, le filet attend.
 narrateur|L'eau avance, goutte après goutte.
 narrateur|Sarah souffle, les épaules baissent.
 papa|C'est à toi, Sarah.
-enfant-f|J'y glisse le citron.
-maman|Chacun son tour, sur l'évier.
+enfant-f|J'y verse le jaune.
+maman|D'abord l'eau, ensuite le citron.
 narrateur|Le filet se tait, enfin.</t>
         </is>
       </c>
@@ -9598,12 +9604,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. Chacun son tour, sur l'évier. Le pichet bleu tient, enfin. Le sucrier blanc garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
+          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. D'abord l'eau, ensuite le jaune. Le pichet bleu tient, enfin. Le sucrier blanc garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. Chacun son tour, sur l'évier. Le pichet bleu tient, enfin. Le sucrier blanc garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
+          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. D'abord l'eau, ensuite le jaune. Le pichet bleu tient, enfin. Le sucrier blanc garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9741,7 +9747,7 @@
           <t>narrateur|Sarah boit, le filet tout calme.
 papa|J'ai ouvert, puis c'était toi.
 enfant-f|J'ai attendu l'eau.
-maman|Chacun son tour, sur l'évier.
+maman|D'abord l'eau, ensuite le jaune.
 narrateur|Le pichet bleu tient, enfin.
 narrateur|Le sucrier blanc garde un grain de lumière.
 narrateur|Sarah souffle dessus, tout doux.
@@ -9773,12 +9779,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, près du sucrier. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Vous avez demandé, et ça marche. Le jus tient tout seul, maintenant. Un carré de carreau reste tiède, autour.</t>
+          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, près du sucrier. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Le jaune tombe, le pichet se remplit. Le jus tient tout seul, maintenant. Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, près du sucrier. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Vous avez demandé, et ça marche. Le jus tient tout seul, maintenant. Un carré de carreau reste tiède, autour.</t>
+          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, près du sucrier. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Le jaune tombe, le pichet se remplit. Le jus tient tout seul, maintenant. Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9919,9 +9925,9 @@
 narrateur|Sarah glisse un grain, les mains calmes.
 narrateur|L'autre main suit, le pichet au calme.
 enfant-f|Toi tu presses, moi je verse.
-maman|Vous avez demandé, et ça marche.
+narrateur|Le jaune tombe, le pichet se remplit.
 papa|Le jus tient tout seul, maintenant.
-narrateur|Un carré de carreau reste tiède, autour.</t>
+narrateur|Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
     </row>
@@ -9948,12 +9954,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. L'entrée du pichet est à vous. L'évier a rendu le calme. Le sucrier blanc garde un grain, au fond. Un rond de chaleur reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
+          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. Le pichet a son jaune, à vous. L'évier a rendu le calme. Le sucrier blanc garde un grain, au fond. Un rond d'eau reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. L'entrée du pichet est à vous. L'évier a rendu le calme. Le sucrier blanc garde un grain, au fond. Un rond de chaleur reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
+          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. Le pichet a son jaune, à vous. L'évier a rendu le calme. Le sucrier blanc garde un grain, au fond. Un rond d'eau reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10091,10 +10097,10 @@
           <t>narrateur|Sarah boit, le citron pressé par papa.
 enfant-f|Tu pressais, tout doux.
 papa|Le jus est tombé, juste assez.
-maman|L'entrée du pichet est à vous.
+maman|Le pichet a son jaune, à vous.
 narrateur|L'évier a rendu le calme.
 narrateur|Le sucrier blanc garde un grain, au fond.
-narrateur|Un rond de chaleur reste sur le carreau.
+narrateur|Un rond d'eau reste sur le carreau.
 enfant-f|Regarde, papa, il brille.
 narrateur|Une odeur de citron reste, au frais.</t>
         </is>
@@ -10123,12 +10129,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Sarah grimpe, le sucrier contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le sucrier vacille, un grain s'envole. Le sucrier blanc n'est plus à sa place. Tes genoux font trop de vagues. Le tabouret n'a pas encore de table. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah grimpe, le sucrier contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le sucrier vacille, un grain s'envole. Le sucrier blanc n'est plus à sa place. Tes genoux font trop de vagues. Le jus n'est pas encore versé. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Sarah grimpe, le sucrier contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le sucrier vacille, un grain s'envole. Le sucrier blanc n'est plus à sa place. Tes genoux font trop de vagues. Le tabouret n'a pas encore de table. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah grimpe, le sucrier contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le sucrier vacille, un grain s'envole. Le sucrier blanc n'est plus à sa place. Tes genoux font trop de vagues. Le jus n'est pas encore versé. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10269,7 +10275,7 @@
 narrateur|Le sucrier vacille, un grain s'envole.
 narrateur|Le sucrier blanc n'est plus à sa place.
 maman|Tes genoux font trop de vagues.
-papa|Le tabouret n'a pas encore de table.
+papa|Le jus n'est pas encore versé.
 enfant-f|On verse comment, alors ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -10490,12 +10496,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>On fait des sauts. Tu rebondis, puis tu verses. Le sucrier voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Vous avez joué, puis versé. Le tabouret est une table, maintenant. Le sucrier blanc a trouvé son coin. La citronnade est là, tout haut.</t>
+          <t>On fait des sauts. Tu rebondis, puis tu verses. Le sucrier voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Sarah verse, le pichet se teinte. Le tabouret est une table, maintenant. Le sucrier blanc reste tout près, en haut. La citronnade est là, tout haut.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>On fait des sauts. Tu rebondis, puis tu verses. Le sucrier voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Vous avez joué, puis versé. Le tabouret est une table, maintenant. Le sucrier blanc a trouvé son coin. La citronnade est là, tout haut.</t>
+          <t>On fait des sauts. Tu rebondis, puis tu verses. Le sucrier voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Sarah verse, le pichet se teinte. Le tabouret est une table, maintenant. Le sucrier blanc reste tout près, en haut. La citronnade est là, tout haut.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10635,9 +10641,9 @@
 narrateur|Le sucrier voyage d'un genou à l'autre.
 narrateur|Le bois penche, puis se tient droit.
 enfant-f|Doucement, les sauts tiennent.
-maman|Vous avez joué, puis versé.
+narrateur|Sarah verse, le pichet se teinte.
 papa|Le tabouret est une table, maintenant.
-narrateur|Le sucrier blanc a trouvé son coin.
+narrateur|Le sucrier blanc reste tout près, en haut.
 enfant-f|La citronnade est là, tout haut.</t>
         </is>
       </c>
@@ -10840,12 +10846,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le sucrier reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Le tabouret a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
+          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le sucrier reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Sarah verse, une goutte, puis l'eau. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le sucrier reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Le tabouret a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
+          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le sucrier reste sage, au creux des mains. Le compte se tait, enfin. Maintenant ! Sarah verse, une goutte, puis l'eau. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -10986,7 +10992,7 @@
 narrateur|Le sucrier reste sage, au creux des mains.
 narrateur|Le compte se tait, enfin.
 enfant-f|Maintenant !
-maman|Le tabouret a fini ses vagues.
+narrateur|Sarah verse, une goutte, puis l'eau.
 papa|Tes genoux se sont assis, eux aussi.
 narrateur|Un pli du torchon retombe, tout lent.</t>
         </is>
@@ -11190,12 +11196,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu portes le pichet ? Je le porte, tout chaud. Papa porte le pichet, près du sucrier. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le tabouret devient une table, tout haut. Vous avez demandé le bord. Ses mains ont tenu le jaune.</t>
+          <t>Papa, tu portes le pichet ? Je le porte, tout droit. Papa porte le pichet, près du sucrier. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le jaune tombe, vu d'en haut. Tu as demandé, je porte. Tes mains ont tenu le bord.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu portes le pichet ? Je le porte, tout chaud. Papa porte le pichet, près du sucrier. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le tabouret devient une table, tout haut. Vous avez demandé le bord. Ses mains ont tenu le jaune.</t>
+          <t>Papa, tu portes le pichet ? Je le porte, tout droit. Papa porte le pichet, près du sucrier. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le jaune tombe, vu d'en haut. Tu as demandé, je porte. Tes mains ont tenu le bord.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11331,14 +11337,14 @@
       <c r="AW58" t="inlineStr">
         <is>
           <t>enfant-f|Papa, tu portes le pichet ?
-papa|Je le porte, tout chaud.
+papa|Je le porte, tout droit.
 narrateur|Papa porte le pichet, près du sucrier.
 narrateur|Sarah écoute les mains, plus que ses pieds.
 maman|Tu verses, et ça tient.
 enfant-f|Moi aussi, j'écoute.
-narrateur|Le tabouret devient une table, tout haut.
-papa|Vous avez demandé le bord.
-maman|Ses mains ont tenu le jaune.</t>
+narrateur|Le jaune tombe, vu d'en haut.
+papa|Tu as demandé, je porte.
+maman|Tes mains ont tenu le bord.</t>
         </is>
       </c>
     </row>
@@ -11365,12 +11371,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Vous avez demandé le bord. Le tabouret a rendu vos pas. Le sucrier blanc garde un grain, au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
+          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Tu as demandé, il a porté. Le tabouret a rendu vos pas. Le sucrier blanc garde un grain, au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Vous avez demandé le bord. Le tabouret a rendu vos pas. Le sucrier blanc garde un grain, au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
+          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Tu as demandé, il a porté. Le tabouret a rendu vos pas. Le sucrier blanc garde un grain, au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11508,7 +11514,7 @@
           <t>narrateur|Sarah boit, le pichet porté par papa.
 enfant-f|J'écoutais tes mains.
 papa|Moi aussi, je portais avec toi.
-maman|Vous avez demandé le bord.
+maman|Tu as demandé, il a porté.
 narrateur|Le tabouret a rendu vos pas.
 narrateur|Le sucrier blanc garde un grain, au fond.
 narrateur|Sarah touche le verre, du bout des doigts.
@@ -11540,12 +11546,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord le pichet bleu. Il est lourd, par le bord. Garde-le là, tout droit. L'eau chante un peu, déjà. Le citron et le sucrier, avec toi. Elle les pose près des carreaux. Les trois affaires avancent avec elle. Le pichet veut son jaune. Ses talons frappent le carreau, trop vite. Le pichet d'abord, il est pris.</t>
+          <t>Sarah prend d'abord le pichet bleu. Il est lourd, par le bord. Garde-le là, tout droit. L'eau chante un peu, déjà. Le citron et le sucrier, avec toi. Elle les pose près des carreaux. Le pichet avance, tout bleu, tout lent. Le pichet veut son jaune. Ses talons frappent le carreau, trop vite. Le pichet d'abord, il est pris.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Sarah prend d'abord le pichet bleu. Il est lourd, par le bord. Garde-le là, tout droit. L'eau chante un peu, déjà. Le citron et le sucrier, avec toi. Elle les pose près des carreaux. Les trois affaires avancent avec elle. Le pichet veut son jaune. Ses talons frappent le carreau, trop vite. Le pichet d'abord, il est pris.</t>
+          <t>Sarah prend d'abord le pichet bleu. Il est lourd, par le bord. Garde-le là, tout droit. L'eau chante un peu, déjà. Le citron et le sucrier, avec toi. Elle les pose près des carreaux. Le pichet avance, tout bleu, tout lent. Le pichet veut son jaune. Ses talons frappent le carreau, trop vite. Le pichet d'abord, il est pris.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -11686,7 +11692,7 @@
 narrateur|L'eau chante un peu, déjà.
 papa|Le citron et le sucrier, avec toi.
 narrateur|Elle les pose près des carreaux.
-narrateur|Les trois affaires avancent avec elle.
+narrateur|Le pichet avance, tout bleu, tout lent.
 enfant-f|Le pichet veut son jaune.
 narrateur|Ses talons frappent le carreau, trop vite.
 papa|Le pichet d'abord, il est pris.</t>
@@ -12274,12 +12280,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le pichet sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le pichet penche, l'eau tremble. Le pichet bleu part trop vite. Tes pieds dansent, déjà. La table n'a pas encore de jus. On presse comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Sarah pose le pichet sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le pichet penche, l'eau tremble. Le pichet bleu part trop vite. Tes pieds dansent, déjà. Le jus n'est pas encore là. On presse comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose le pichet sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le pichet penche, l'eau tremble. Le pichet bleu part trop vite. Tes pieds dansent, déjà. La table n'a pas encore de jus. On presse comment, alors ? Tu fais comment, avec nous ?</t>
+          <t>Sarah pose le pichet sur la toile cirée. Ses talons tambourinent le carreau. La citronnade, c'est là, papa ! Le pichet penche, l'eau tremble. Le pichet bleu part trop vite. Tes pieds dansent, déjà. Le jus n'est pas encore là. On presse comment, alors ? Tu fais comment, avec nous ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12420,7 +12426,7 @@
 narrateur|Le pichet penche, l'eau tremble.
 enfant-f|Le pichet bleu part trop vite.
 maman|Tes pieds dansent, déjà.
-papa|La table n'a pas encore de jus.
+papa|Le jus n'est pas encore là.
 enfant-f|On presse comment, alors ?
 papa|Tu fais comment, avec nous ?</t>
         </is>
@@ -12641,12 +12647,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le pichet devient un lac. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Vous avez joué, puis posé. La toile redevient une table, tout douce.</t>
+          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le pichet devient un lac. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Le jus tombe dans le pichet, tout jaune. Tu as roulé, moi j'ai rattrapé. La toile redevient une table, tout douce.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le pichet devient un lac. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Vous avez joué, puis posé. La toile redevient une table, tout douce.</t>
+          <t>On joue à la balle jaune. Toi tu roules, moi je rattrape. Sarah roule, le pichet devient un lac. Le jaune va, revient, sent plus fort. Sarah roule encore, puis s'arrête. La balle est fatiguée. On peut presser, maintenant. Le jus tombe dans le pichet, tout jaune. Tu as roulé, moi j'ai rattrapé. La toile redevient une table, tout douce.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12788,7 +12794,8 @@
 narrateur|Sarah roule encore, puis s'arrête.
 enfant-f|La balle est fatiguée.
 maman|On peut presser, maintenant.
-papa|Vous avez joué, puis posé.
+narrateur|Le jus tombe dans le pichet, tout jaune.
+papa|Tu as roulé, moi j'ai rattrapé.
 narrateur|La toile redevient une table, tout douce.</t>
         </is>
       </c>
@@ -12816,12 +12823,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le pichet bleu garde une goutte, tout au fond. Un grain sucré dort sur la toile. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
+          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le pichet bleu garde une goutte, tout au fond. Sarah lèche une goutte sur le bord. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le pichet bleu garde une goutte, tout au fond. Un grain sucré dort sur la toile. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
+          <t>Sarah boit près de la table, tout petit. La balle est devenue du jus. Tu roulais, moi je rattrapais. Le pichet a son jaune, maintenant. La toile cirée garde un grain sucré. Le pichet bleu garde une goutte, tout au fond. Sarah lèche une goutte sur le bord. Encore une gorgée, papa. La vitre tient encore le soleil.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12962,7 +12969,7 @@
 maman|Le pichet a son jaune, maintenant.
 narrateur|La toile cirée garde un grain sucré.
 narrateur|Le pichet bleu garde une goutte, tout au fond.
-narrateur|Un grain sucré dort sur la toile.
+narrateur|Sarah lèche une goutte sur le bord.
 enfant-f|Encore une gorgée, papa.
 narrateur|La vitre tient encore le soleil.</t>
         </is>
@@ -12991,12 +12998,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>On attend le grain. Sarah pose les genoux au carreau. Le pichet repose, l'eau calme. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. La citronnade peut venir.</t>
+          <t>On attend le grain. Sarah pose les genoux au carreau. Le pichet repose, l'eau calme. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. Le jus tombe, une goutte, puis deux. La citronnade peut venir.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>On attend le grain. Sarah pose les genoux au carreau. Le pichet repose, l'eau calme. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. La citronnade peut venir.</t>
+          <t>On attend le grain. Sarah pose les genoux au carreau. Le pichet repose, l'eau calme. Un grain glisse, puis plus. Il ne bouge plus ? La toile est calme, oui. Tes pieds se sont assis, eux aussi. Sarah presse, tout droit, tout petit. Le jus tombe, une goutte, puis deux. La citronnade peut venir.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13139,6 +13146,7 @@
 maman|La toile est calme, oui.
 papa|Tes pieds se sont assis, eux aussi.
 narrateur|Sarah presse, tout droit, tout petit.
+narrateur|Le jus tombe, une goutte, puis deux.
 enfant-f|La citronnade peut venir.</t>
         </is>
       </c>
@@ -13341,12 +13349,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le pichet, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Vous avez demandé, et ça tient. Ma main fait le bol, ici. La table garde un grain, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le pichet, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Le jus rejoint le sucre, tout jaune. Ma main tient, la tienne verse. La table garde un grain, tout mince.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le pichet, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Vous avez demandé, et ça tient. Ma main fait le bol, ici. La table garde un grain, tout mince.</t>
+          <t>Maman, tu tiens, s'il te plaît ? Je tiens, tu verses le sucre. Maman tient le pichet, Sarah verse. Sarah verse un grain, puis un autre. Le jaune reste sage, dans sa main. Toi tu tiens, moi je verse. Le jus rejoint le sucre, tout jaune. Ma main tient, la tienne verse. La table garde un grain, tout mince.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13487,8 +13495,8 @@
 narrateur|Sarah verse un grain, puis un autre.
 narrateur|Le jaune reste sage, dans sa main.
 enfant-f|Toi tu tiens, moi je verse.
-papa|Vous avez demandé, et ça tient.
-maman|Ma main fait le bol, ici.
+narrateur|Le jus rejoint le sucre, tout jaune.
+maman|Ma main tient, la tienne verse.
 narrateur|La table garde un grain, tout mince.</t>
         </is>
       </c>
@@ -13516,12 +13524,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Vous avez demandé, et ça tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le pichet bleu pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
+          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Tu demandais, maman tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le pichet bleu pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Vous avez demandé, et ça tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le pichet bleu pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
+          <t>Sarah boit, la main de maman tout près. Tu tenais le fruit. Tu demandais, maman tenait. Ma main a fait le bol. La cuisine rend le silence, tout doux. Le pichet bleu pose un grain de lumière. Sarah touche la toile, du bout. Il est à nous. Un rai de soleil barre encore la toile.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13658,7 +13666,7 @@
         <is>
           <t>narrateur|Sarah boit, la main de maman tout près.
 enfant-f|Tu tenais le fruit.
-papa|Vous avez demandé, et ça tenait.
+papa|Tu demandais, maman tenait.
 maman|Ma main a fait le bol.
 narrateur|La cuisine rend le silence, tout doux.
 narrateur|Le pichet bleu pose un grain de lumière.
@@ -13691,12 +13699,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le pichet vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le pichet claque le rebord, trop fort. Une goutte rebondit, puis s'en va. Ton corps veut encore courir. L'évier n'a pas encore de pichet. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah porte le pichet vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le pichet claque le rebord, trop fort. Une goutte rebondit, puis s'en va. Tes genoux rebondissent encore. Le pichet n'a pas encore de jus. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le pichet vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le pichet claque le rebord, trop fort. Une goutte rebondit, puis s'en va. Ton corps veut encore courir. L'évier n'a pas encore de pichet. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah porte le pichet vers l'eau. Ici, le jus va tomber, maman. Ses genoux font un petit trampoline. Le pichet claque le rebord, trop fort. Une goutte rebondit, puis s'en va. Tes genoux rebondissent encore. Le pichet n'a pas encore de jus. On peut jouer avec, quand même ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13836,8 +13844,8 @@
 narrateur|Ses genoux font un petit trampoline.
 narrateur|Le pichet claque le rebord, trop fort.
 narrateur|Une goutte rebondit, puis s'en va.
-maman|Ton corps veut encore courir.
-papa|L'évier n'a pas encore de pichet.
+maman|Tes genoux rebondissent encore.
+papa|Le pichet n'a pas encore de jus.
 enfant-f|On peut jouer avec, quand même ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -14058,12 +14066,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le pichet, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Vous avez joué, puis posé le fruit. L'évier est devenu un ruisseau. Le pichet bleu a trouvé son coin. Le jus est là, tout bas.</t>
+          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le pichet, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Le pichet se teinte, tout doucement. L'évier est devenu un ruisseau. Le pichet bleu reste près de l'eau. Le jus est là, tout bas.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le pichet, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Vous avez joué, puis posé le fruit. L'évier est devenu un ruisseau. Le pichet bleu a trouvé son coin. Le jus est là, tout bas.</t>
+          <t>On fait des gouttes. Toi tu presses, moi je compte. Sarah penche le pichet, papa compte. Des perles tombent, une après l'autre. La dernière est au bout. Le pichet se teinte, tout doucement. L'évier est devenu un ruisseau. Le pichet bleu reste près de l'eau. Le jus est là, tout bas.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14203,9 +14211,9 @@
 narrateur|Sarah penche le pichet, papa compte.
 narrateur|Des perles tombent, une après l'autre.
 enfant-f|La dernière est au bout.
-maman|Vous avez joué, puis posé le fruit.
+narrateur|Le pichet se teinte, tout doucement.
 papa|L'évier est devenu un ruisseau.
-narrateur|Le pichet bleu a trouvé son coin.
+narrateur|Le pichet bleu reste près de l'eau.
 enfant-f|Le jus est là, tout bas.</t>
         </is>
       </c>
@@ -14408,12 +14416,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>J'attends le filet. Moi je l'ouvre, puis c'est toi. Sarah tient le pichet, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y glisse le citron. Chacun son tour, sur l'évier. Le filet se tait, enfin.</t>
+          <t>J'attends le filet. Moi j'ouvre un peu, puis c'est toi. Sarah tient le pichet, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y verse le jaune. D'abord l'eau, ensuite le citron. Le filet se tait, enfin.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>J'attends le filet. Moi je l'ouvre, puis c'est toi. Sarah tient le pichet, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y glisse le citron. Chacun son tour, sur l'évier. Le filet se tait, enfin.</t>
+          <t>J'attends le filet. Moi j'ouvre un peu, puis c'est toi. Sarah tient le pichet, le filet attend. L'eau avance, goutte après goutte. Sarah souffle, les épaules baissent. C'est à toi, Sarah. J'y verse le jaune. D'abord l'eau, ensuite le citron. Le filet se tait, enfin.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14549,13 +14557,13 @@
       <c r="AW76" t="inlineStr">
         <is>
           <t>enfant-f|J'attends le filet.
-papa|Moi je l'ouvre, puis c'est toi.
+papa|Moi j'ouvre un peu, puis c'est toi.
 narrateur|Sarah tient le pichet, le filet attend.
 narrateur|L'eau avance, goutte après goutte.
 narrateur|Sarah souffle, les épaules baissent.
 papa|C'est à toi, Sarah.
-enfant-f|J'y glisse le citron.
-maman|Chacun son tour, sur l'évier.
+enfant-f|J'y verse le jaune.
+maman|D'abord l'eau, ensuite le citron.
 narrateur|Le filet se tait, enfin.</t>
         </is>
       </c>
@@ -14583,12 +14591,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. Chacun son tour, sur l'évier. Le pichet bleu tient, enfin. Le pichet bleu garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
+          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. D'abord l'eau, ensuite le jaune. Le pichet bleu tient, enfin. Le pichet bleu garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. Chacun son tour, sur l'évier. Le pichet bleu tient, enfin. Le pichet bleu garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
+          <t>Sarah boit, le filet tout calme. J'ai ouvert, puis c'était toi. J'ai attendu l'eau. D'abord l'eau, ensuite le jaune. Le pichet bleu tient, enfin. Le pichet bleu garde un grain de lumière. Sarah souffle dessus, tout doux. Ça pique, puis c'est doux. Un fil d'eau sèche contre le rebord.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14726,7 +14734,7 @@
           <t>narrateur|Sarah boit, le filet tout calme.
 papa|J'ai ouvert, puis c'était toi.
 enfant-f|J'ai attendu l'eau.
-maman|Chacun son tour, sur l'évier.
+maman|D'abord l'eau, ensuite le jaune.
 narrateur|Le pichet bleu tient, enfin.
 narrateur|Le pichet bleu garde un grain de lumière.
 narrateur|Sarah souffle dessus, tout doux.
@@ -14758,12 +14766,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, au-dessus du pichet. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Vous avez demandé, et ça marche. Le jus tient tout seul, maintenant. Un carré de carreau reste tiède, autour.</t>
+          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, au-dessus du pichet. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Le jaune tombe, le pichet se remplit. Le jus tient tout seul, maintenant. Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, au-dessus du pichet. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Vous avez demandé, et ça marche. Le jus tient tout seul, maintenant. Un carré de carreau reste tiède, autour.</t>
+          <t>Papa, tu presses le citron ? Je le presse, tout doux. Papa presse, au-dessus du pichet. Sarah glisse un grain, les mains calmes. L'autre main suit, le pichet au calme. Toi tu presses, moi je verse. Le jaune tombe, le pichet se remplit. Le jus tient tout seul, maintenant. Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14904,9 +14912,9 @@
 narrateur|Sarah glisse un grain, les mains calmes.
 narrateur|L'autre main suit, le pichet au calme.
 enfant-f|Toi tu presses, moi je verse.
-maman|Vous avez demandé, et ça marche.
+narrateur|Le jaune tombe, le pichet se remplit.
 papa|Le jus tient tout seul, maintenant.
-narrateur|Un carré de carreau reste tiède, autour.</t>
+narrateur|Un carré de carreau reste froid, autour.</t>
         </is>
       </c>
     </row>
@@ -14933,12 +14941,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. L'entrée du pichet est à vous. L'évier a rendu le calme. Le pichet bleu garde une goutte, tout au fond. Un rond de chaleur reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
+          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. Le pichet a son jaune, à vous. L'évier a rendu le calme. Le pichet bleu garde une goutte, tout au fond. Un rond d'eau reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. L'entrée du pichet est à vous. L'évier a rendu le calme. Le pichet bleu garde une goutte, tout au fond. Un rond de chaleur reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
+          <t>Sarah boit, le citron pressé par papa. Tu pressais, tout doux. Le jus est tombé, juste assez. Le pichet a son jaune, à vous. L'évier a rendu le calme. Le pichet bleu garde une goutte, tout au fond. Un rond d'eau reste sur le carreau. Regarde, papa, il brille. Une odeur de citron reste, au frais.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15076,10 +15084,10 @@
           <t>narrateur|Sarah boit, le citron pressé par papa.
 enfant-f|Tu pressais, tout doux.
 papa|Le jus est tombé, juste assez.
-maman|L'entrée du pichet est à vous.
+maman|Le pichet a son jaune, à vous.
 narrateur|L'évier a rendu le calme.
 narrateur|Le pichet bleu garde une goutte, tout au fond.
-narrateur|Un rond de chaleur reste sur le carreau.
+narrateur|Un rond d'eau reste sur le carreau.
 enfant-f|Regarde, papa, il brille.
 narrateur|Une odeur de citron reste, au frais.</t>
         </is>
@@ -15108,12 +15116,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Sarah grimpe, le pichet contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le pichet penche, l'eau fait une vague. Le pichet bleu n'est plus à sa place. Tes genoux font trop de vagues. Le tabouret n'a pas encore de table. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah grimpe, le pichet contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le pichet penche, l'eau fait une vague. Le pichet bleu n'est plus à sa place. Tes genoux font trop de vagues. Le jus n'est pas encore versé. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Sarah grimpe, le pichet contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le pichet penche, l'eau fait une vague. Le pichet bleu n'est plus à sa place. Tes genoux font trop de vagues. Le tabouret n'a pas encore de table. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
+          <t>Sarah grimpe, le pichet contre elle. Ici, je suis grande, papa. Le bois du tabouret rend chaque pas. Le pichet penche, l'eau fait une vague. Le pichet bleu n'est plus à sa place. Tes genoux font trop de vagues. Le jus n'est pas encore versé. On verse comment, alors ? Vous trouvez, tous les trois ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15254,7 +15262,7 @@
 narrateur|Le pichet penche, l'eau fait une vague.
 narrateur|Le pichet bleu n'est plus à sa place.
 maman|Tes genoux font trop de vagues.
-papa|Le tabouret n'a pas encore de table.
+papa|Le jus n'est pas encore versé.
 enfant-f|On verse comment, alors ?
 papa|Vous trouvez, tous les trois ?</t>
         </is>
@@ -15475,12 +15483,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>On fait des sauts. Tu rebondis, puis tu verses. Le pichet voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Vous avez joué, puis versé. Le tabouret est une table, maintenant. Le pichet bleu a trouvé son coin. La citronnade est là, tout haut.</t>
+          <t>On fait des sauts. Tu rebondis, puis tu verses. Le pichet voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Sarah verse, le pichet se teinte. Le tabouret est une table, maintenant. Le pichet bleu reste tout près, en haut. La citronnade est là, tout haut.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>On fait des sauts. Tu rebondis, puis tu verses. Le pichet voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Vous avez joué, puis versé. Le tabouret est une table, maintenant. Le pichet bleu a trouvé son coin. La citronnade est là, tout haut.</t>
+          <t>On fait des sauts. Tu rebondis, puis tu verses. Le pichet voyage d'un genou à l'autre. Le bois penche, puis se tient droit. Doucement, les sauts tiennent. Sarah verse, le pichet se teinte. Le tabouret est une table, maintenant. Le pichet bleu reste tout près, en haut. La citronnade est là, tout haut.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15620,9 +15628,9 @@
 narrateur|Le pichet voyage d'un genou à l'autre.
 narrateur|Le bois penche, puis se tient droit.
 enfant-f|Doucement, les sauts tiennent.
-maman|Vous avez joué, puis versé.
+narrateur|Sarah verse, le pichet se teinte.
 papa|Le tabouret est une table, maintenant.
-narrateur|Le pichet bleu a trouvé son coin.
+narrateur|Le pichet bleu reste tout près, en haut.
 enfant-f|La citronnade est là, tout haut.</t>
         </is>
       </c>
@@ -15825,12 +15833,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le pichet reste sage, au creux des genoux. Le compte se tait, enfin. Maintenant ! Le tabouret a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
+          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le pichet reste sage, au creux des genoux. Le compte se tait, enfin. Maintenant ! Sarah verse, une goutte, puis l'eau. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le pichet reste sage, au creux des genoux. Le compte se tait, enfin. Maintenant ! Le tabouret a fini ses vagues. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
+          <t>On attend le compte. Un, deux, trois, tu verses. Un saut, puis le bois reste calme. Le pichet reste sage, au creux des genoux. Le compte se tait, enfin. Maintenant ! Sarah verse, une goutte, puis l'eau. Tes genoux se sont assis, eux aussi. Un pli du torchon retombe, tout lent.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15971,7 +15979,7 @@
 narrateur|Le pichet reste sage, au creux des genoux.
 narrateur|Le compte se tait, enfin.
 enfant-f|Maintenant !
-maman|Le tabouret a fini ses vagues.
+narrateur|Sarah verse, une goutte, puis l'eau.
 papa|Tes genoux se sont assis, eux aussi.
 narrateur|Un pli du torchon retombe, tout lent.</t>
         </is>
@@ -16175,12 +16183,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu portes le pichet ? Je le porte, tout chaud. Papa porte le pichet, tout droit. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le tabouret devient une table, tout haut. Vous avez demandé le bord. Ses mains ont tenu le jaune.</t>
+          <t>Papa, tu portes le pichet ? Je le porte, tout droit. Papa porte le pichet, tout droit. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le jaune tombe, vu d'en haut. Tu as demandé, je porte. Tes mains ont tenu le bord.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu portes le pichet ? Je le porte, tout chaud. Papa porte le pichet, tout droit. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le tabouret devient une table, tout haut. Vous avez demandé le bord. Ses mains ont tenu le jaune.</t>
+          <t>Papa, tu portes le pichet ? Je le porte, tout droit. Papa porte le pichet, tout droit. Sarah écoute les mains, plus que ses pieds. Tu verses, et ça tient. Moi aussi, j'écoute. Le jaune tombe, vu d'en haut. Tu as demandé, je porte. Tes mains ont tenu le bord.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16316,14 +16324,14 @@
       <c r="AW86" t="inlineStr">
         <is>
           <t>enfant-f|Papa, tu portes le pichet ?
-papa|Je le porte, tout chaud.
+papa|Je le porte, tout droit.
 narrateur|Papa porte le pichet, tout droit.
 narrateur|Sarah écoute les mains, plus que ses pieds.
 maman|Tu verses, et ça tient.
 enfant-f|Moi aussi, j'écoute.
-narrateur|Le tabouret devient une table, tout haut.
-papa|Vous avez demandé le bord.
-maman|Ses mains ont tenu le jaune.</t>
+narrateur|Le jaune tombe, vu d'en haut.
+papa|Tu as demandé, je porte.
+maman|Tes mains ont tenu le bord.</t>
         </is>
       </c>
     </row>
@@ -16350,12 +16358,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Vous avez demandé le bord. Le tabouret a rendu vos pas. Le pichet bleu garde une goutte, tout au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
+          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Tu as demandé, il a porté. Le tabouret a rendu vos pas. Le pichet bleu garde une goutte, tout au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Vous avez demandé le bord. Le tabouret a rendu vos pas. Le pichet bleu garde une goutte, tout au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
+          <t>Sarah boit, le pichet porté par papa. J'écoutais tes mains. Moi aussi, je portais avec toi. Tu as demandé, il a porté. Le tabouret a rendu vos pas. Le pichet bleu garde une goutte, tout au fond. Sarah touche le verre, du bout des doigts. Il est à nous, maman. Le bleu garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16493,7 +16501,7 @@
           <t>narrateur|Sarah boit, le pichet porté par papa.
 enfant-f|J'écoutais tes mains.
 papa|Moi aussi, je portais avec toi.
-maman|Vous avez demandé le bord.
+maman|Tu as demandé, il a porté.
 narrateur|Le tabouret a rendu vos pas.
 narrateur|Le pichet bleu garde une goutte, tout au fond.
 narrateur|Sarah touche le verre, du bout des doigts.
@@ -16519,7 +16527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16562,6 +16570,20 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>